<commit_message>
Ganti istilah Kursus menjadi Mapel / Mata Pelajaran
Label singkat memakai "Mapel" (Mapel Saya, Katalog Mapel, Mapel baru),
kalimat memakai "mata pelajaran". Berlaku di tampilan, pesan backend,
panduan, dan templat Excel impor siswa. Backend v2.0.1, tampilan v2.0.2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013X3wAQ8LbjfZLFJvCAeUBB
</commit_message>
<xml_diff>
--- a/templates/Templat-Impor-Siswa.xlsx
+++ b/templates/Templat-Impor-Siswa.xlsx
@@ -219,7 +219,7 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>Mis. X TJKT 1. Dipakai untuk mendaftarkan satu kelas sekaligus ke kursus.</t>
+        <t>Mis. X TJKT 1. Dipakai untuk mendaftarkan satu kelas sekaligus ke mata pelajaran.</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -239,7 +239,7 @@
     </comment>
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>siswa / guru / admin. Kosong = siswa. (Diabaikan saat guru mengimpor ke kursus.)</t>
+        <t>siswa / guru / admin. Kosong = siswa. (Diabaikan saat guru mengimpor ke mapel.)</t>
       </text>
     </comment>
   </commentList>
@@ -4260,14 +4260,14 @@
     <row r="8" ht="30" customHeight="1">
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>5.  Baris dengan username yang sudah terdaftar akan dilewati (admin) atau langsung didaftarkan ke kursus (impor dari halaman Peserta).</t>
+          <t>5.  Baris dengan username yang sudah terdaftar akan dilewati (admin) atau langsung didaftarkan ke mata pelajaran (impor dari halaman Peserta).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>6.  Simpan sebagai .xlsx, lalu unggah di LMS: Administrasi Situs → Pengguna → Impor, atau di kursus: Peserta → Impor Excel.</t>
+          <t>6.  Simpan sebagai .xlsx, lalu unggah di LMS: Administrasi Situs → Pengguna → Impor, atau di halaman Mapel: Peserta → Impor Excel.</t>
         </is>
       </c>
     </row>

</xml_diff>